<commit_message>
docs: refresh enhancement status workbook for spec v2
Adds the 8 new items from the (1) version of the spec (upload subtitle,
all-closed accordions, recategorize inputs with A/B subsections, hide
Workforce Protection in target mode + flip toggle, bottom nav arrows).

Totals: 26 Done, 6 Deferred, 1 Info, 33 items total.
</commit_message>
<xml_diff>
--- a/docs/150526_enhancement_status.xlsx
+++ b/docs/150526_enhancement_status.xlsx
@@ -518,14 +518,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -573,7 +573,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Placeholder cpc-logo.png still in place; awaiting hi-res asset from Saad. Logo plumbing already in place at both desktop/src/features/HomePage.tsx and desktop/src/features/AppShell.tsx (sidebar footer).</t>
+          <t>Placeholder cpc-logo.png in place; awaiting hi-res asset from Saad. Logo slots ready at desktop/src/features/HomePage.tsx and the sidebar footer in AppShell.tsx.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Net-new workflow stage. Open questions: position in flow (before or after upload?), backend support, multi-tenant data persistence per BU.</t>
+          <t>Net-new workflow stage. See the Open discussion sheet for the open questions.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Removed Workforce Studio label and alt text. Logo moved from sidebar header to sidebar footer (above engine status).</t>
+          <t>Removed Workforce Studio label and alt. Logo moved from sidebar header to sidebar footer above engine status.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Data Upload — Remove 'Upload workbook' from left-panel bottom</t>
+          <t>Data Upload — Before upload, change subtitle to 'Upload In-house and Outsourced Employees Payroll in one [Excel workbook]'</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -708,12 +708,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Button label shortened: 'Upload workbook' / 'Upload new workbook' → 'Upload' / 'Upload new'.</t>
+          <t>Subtitle updated. Final wording uses 'Excel workbook' rather than 'XLS file' because the app accepts .xlsx only (modern OOXML); .xls (legacy BIFF) is rejected by the validator.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>commit 1 / AppShell.tsx</t>
+          <t>commits 8 + 11 / UploadWorkspace.tsx</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Data Upload — After upload, single 'Data Loaded' message (not duplicate 'workbook loaded')</t>
+          <t>Data Upload — Remove 'Upload workbook' from left-panel bottom</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -735,12 +735,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Section eyebrow renamed to 'Data Loaded'. Subtitle row replaced with the loaded workbook filename so the header is informative without duplication.</t>
+          <t>Button label shortened: 'Upload workbook' / 'Upload new workbook' → 'Upload' / 'Upload new'.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>commit 2 / UploadWorkspace.tsx</t>
+          <t>commit 1 / AppShell.tsx</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Data Upload — Rename 'Subcontracted' → 'Outsourced'</t>
+          <t>Data Upload — After upload, single 'Data Loaded' message (not duplicate 'workbook loaded')</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>UI label updated on the metric card. NOT changed: the Excel SHEET NAME 'Subcontractor' (user file format requirement) and internal API field names (would break client compatibility).</t>
+          <t>Section eyebrow renamed to 'Data Loaded'. Subtitle row replaced with the loaded workbook filename so the header is informative without duplication.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Data Upload — Reorganize boxes (total full width on top, then in-house / outsourced / job families row)</t>
+          <t>Data Upload — Rename 'Subcontracted' → 'Outsourced'</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -789,12 +789,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>New data-health-total class for the full-width total card; data-health-grid--triple for the 3-card row below.</t>
+          <t>UI label updated on the metric card. NOT changed: the Excel SHEET NAME 'Subcontractor' (user file format requirement) and internal API field names (would break client compatibility).</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>commit 2 / UploadWorkspace.tsx + styles.css</t>
+          <t>commit 2 / UploadWorkspace.tsx</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Additional Inputs — No need for 'Brand new' on this sheet</t>
+          <t>Data Upload — Reorganize boxes (total full width on top, then in-house / outsourced / job families row)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>All 'brand-new family' wording stripped from button labels, wizard titles, and metadata rows.</t>
+          <t>New data-health-total class for the full-width total card; data-health-grid--triple for the 3-card row below.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>commit 3 / MappingResolveWorkspace.tsx</t>
+          <t>commit 2 / UploadWorkspace.tsx + styles.css</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Additional Inputs — Add 'Job' to all 'families' (Add a Job Family, Name of job family, etc.)</t>
+          <t>Additional Inputs — No need for 'Brand new' on this sheet</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Custom families → Custom job families. Family name → Name of job family. Edit family → Edit job family. Define family from selected → Define job family from selected.</t>
+          <t>All 'brand-new family' wording stripped from button labels, wizard titles, and metadata rows.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -860,22 +860,22 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Additional Inputs — '1 Custom' badge persistence across app restarts?</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Answered (info)</t>
+          <t>Additional Inputs — Add 'Job' to all 'families'</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Desktop React ALREADY persists custom families across restarts via localStorage (see App.tsx persistGet/persistSet on 'custom_families'). Streamlit is session-only — Streamlit was out of scope for this PR so no change there.</t>
+          <t>Custom families → Custom job families. Family name → Name of job family. Edit family → Edit job family. Define family from selected → Define job family from selected.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>commit 3 / MappingResolveWorkspace.tsx</t>
         </is>
       </c>
     </row>
@@ -887,22 +887,22 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>User Assumption — No workbook/data-loaded window on top</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Additional Inputs — '1 Custom' badge persistence across app restarts?</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Answered (info)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Upload metrics card no longer renders on the Ready (User Assumptions) stage; UploadWorkspace is now upload-stage-only.</t>
+          <t>Desktop React ALREADY persists custom families across restarts via localStorage (App.tsx persistGet/persistSet on 'custom_families'). Streamlit is session-only — Streamlit out of scope for this PR.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>commit 2 / App.tsx</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>User Assumption — Drop repeated 'User assumptions'; just 'Optimization Mode' with two radio options</t>
+          <t>User Assumption — No workbook/data-loaded window on top</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -924,12 +924,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>In-content 'User Assumptions' eyebrow removed; the topbar's 'USER ASSUMPTIONS' green tab title remains as the single source of truth. Two-mode toggle preserved.</t>
+          <t>Upload metrics card no longer renders on the Ready stage; UploadWorkspace is upload-stage-only.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>commit 4 / ScenarioControls.tsx</t>
+          <t>commit 2 / App.tsx</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>User Assumption — If Target plan selected, show Target Manpower Plan window</t>
+          <t>User Assumption — Drop repeated 'User assumptions'; just 'Optimization Mode' with two radio options</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -951,12 +951,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Already conditional (isTargetMode). Verified after the User Assumptions header cleanup. Auto-opens the target accordion when the mode toggles.</t>
+          <t>In-content 'User Assumptions' eyebrow removed; the topbar's 'USER ASSUMPTIONS' tab title is the single source of truth.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>no change needed</t>
+          <t>commit 4 / ScenarioControls.tsx</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>All Tabs — Remove second row in upper white strip; keep title in green, larger</t>
+          <t>User Assumption — If Target plan selected, show Target Manpower Plan window</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -978,51 +978,51 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Topbar collapses to a single row. Green eyebrow promoted to a 22px display-font heading; subtitle row removed. Same treatment across Data Upload / Additional Inputs / User Assumptions / Output.</t>
+          <t>Already conditional (isTargetMode). Verified after the User Assumptions header cleanup. Auto-opens the target accordion when the mode toggles.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>commit 1 / AppShell.tsx + styles.css</t>
+          <t>no change needed</t>
         </is>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>After homepage — list of companies with 'to be configured', click MGIC; tab 'BU Selection'</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Deferred (discussion)</t>
+          <t>User Assumption — Rename 'Assumption and Input' section to just 'Inputs'</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Same as the Look &amp; Feel BU Selection entry — net-new stage that needs a design pass. Risk noted: tool currently assumes one BU per laptop.</t>
+          <t>The inner SectionHeader for the inputs panel was reduced to title='Inputs' (no eyebrow). The 'Assumptions' eyebrow disappeared in commit 4.</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>follow-up PR</t>
+          <t>commit 4 / ScenarioControls.tsx</t>
         </is>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Reduce processing time after upload</t>
+          <t>User Assumption — All input windows closed by default (no first one open)</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1032,78 +1032,78 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>94.06s → 19.25s on Manpower.xlsx (~4.9× faster). Root cause: normalize_lookup_text called 16.3M times and per-row dict rebuilds in get_numeric_from_row. Fix: lru_cache + hoist the per-DataFrame column resolver. Cache hit rate 99.94%. All tests still pass.</t>
+          <t>openSections initial state set to new Set(); user can scan all category headings before opening any. Target Manpower Plan still auto-opens when target mode is selected.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>commit 7 / manpower_app/utils.py</t>
+          <t>commit 8 / ScenarioControls.tsx</t>
         </is>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>After XLS processing — why is 'add a job family' visible? (discuss)</t>
+          <t>User Assumption — Recategorize inputs: (1) Saudization, (2) Outsourced Employees, (3) Workforce Protection</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Done (resolved by hiding outside Target mode)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Button now only appears when 'Input and Optimize a Target Manpower Plan' is selected, with a short hint explaining the flow. In Current mode it's hidden — a family with no payroll rows has nothing to optimize.</t>
+          <t>Replaced the previous (Saudization &amp; Risk) + (Workforce Protection) + (Advanced Settings) layout with the three top-level categories. Hard Inputs (ratio overrides) remains as a separate fourth accordion.</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>commit 6 / MappingResolveWorkspace.tsx + App.tsx</t>
+          <t>commit 9 / ScenarioControls.tsx</t>
         </is>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Make Outsourceable / Fully Inhouse / Partially Outsourceable dynamic</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Deferred (discussion)</t>
+          <t>User Assumption — Saudization subsections: A) Overall, B) By Job Family (side-by-side)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Currently hardcoded in manpower_app/rules.py (OUTSOURCEABILITY_RULES dict). Open question: source for dynamic values — workbook column, in-app editor, or both? Affects rules, costs, optimization constraints. Backend rework required.</t>
+          <t>Two-column grid (.scenario-two-column, collapses to 1 column under 980px). A = enforce + overall rate + Saudi cost premium. B = engineer/sales/management rates.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>follow-up PR</t>
+          <t>commit 9 / ScenarioControls.tsx + styles.css</t>
         </is>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tool should handle Saudis-cheaper-than-non-Saudis (auto-correct)</t>
+          <t>User Assumption — Outsourced Employees subsections: A) Risk Factor with (ⓘ) tooltip, B) Renegotiated Rate (side-by-side)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1113,78 +1113,78 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Saudi cost premium floored at 1.0× in three places (defense in depth): desktop slider min, manpower_api Pydantic validator, and manpower_app.costs.calculate_inhouse_cost_split. Saudis can no longer be configured as cheaper than non-Saudis from any code path.</t>
+          <t>A = risk factor slider with an info pill explaining the haircut math. B = negotiated-rates toggle reveals insurance/service margin, plus Override outsource cost + discount slider (moved here from Advanced).</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>commit 4 / costs.py + ScenarioControls.tsx + app.py</t>
+          <t>commit 9 / ScenarioControls.tsx + styles.css</t>
         </is>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Hard inputs — edit ratio AND driver name (e.g., quarries labor vs quarries skilled labor)</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Deferred (discussion)</t>
+          <t>User Assumption — Workforce Protection: hide in Target mode; rename + flip 'Allow reducing Saudi headcount' → 'Protect Current Saudis'</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Driver mappings are hardcoded in manpower_app/ratios.py:calculate_driver_values. Making this user-editable needs the same backend pattern as the dynamic-outsourceability item: new settings field, new API contract, propagation through the LP. Best done with #20.</t>
+          <t>Accordion is hidden entirely when optimization_mode === 'target'. Toggle label is renamed and the semantics are inverted: checked = protect (the safer default). Parallel to 'Protect tenured employees' below.</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>follow-up PR</t>
+          <t>commits 8 + 9 / ScenarioControls.tsx</t>
         </is>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Target plan — ask about drivers so ratios can be recalculated</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Deferred (discussion)</t>
+          <t>All Tabs — Bottom navigation arrows (Prev / Next)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Depends on the editable-driver work (#22). Once a user can pin which profession is the ratio driver, the target plan UI needs an input for the driver headcount.</t>
+          <t>StageNav component at the foot of each content stage. Buttons disable when the prev/next stage is unreachable. Labels show the destination stage rather than just an arrow.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>follow-up PR</t>
+          <t>commit 10 / AppShell.tsx + styles.css</t>
         </is>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Debugging</t>
+          <t>Look &amp; Feel</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Risk input slider — should reach zero</t>
+          <t>All Tabs — Remove second row in upper white strip; keep title in green, larger</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -1194,37 +1194,253 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Slider min lowered from 0.01 to 0 in both UI (ScenarioControls.tsx) and API (Pydantic gt=0 → ge=0). At R=0 the LP constraint degenerates cleanly to O+I ≥ M; the rearranged closed-form (T−M)/R is only consulted when R&gt;0. README updated.</t>
+          <t>Topbar collapses to a single row. Green eyebrow promoted to a 22px display-font heading; subtitle row removed.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>commit 4 / ScenarioControls.tsx + app.py + README.md</t>
+          <t>commit 1 / AppShell.tsx + styles.css</t>
         </is>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>After homepage — list of companies; click MGIC; tab 'BU Selection'</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Deferred (discussion)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Net-new stage that needs a design pass. Risk noted in the spec: tool currently assumes one BU per laptop.</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>follow-up PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Reduce processing time after upload</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>94.06s → 19.25s on Manpower.xlsx (~4.9× faster). Root cause: normalize_lookup_text called 16.3M times and per-row dict rebuilds in get_numeric_from_row. Fix: lru_cache + hoist the per-DataFrame column resolver. Cache hit rate 99.94%. All tests still pass. Remaining cost is pandas .apply row iteration + openpyxl XML parsing — bigger refactors deferred.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>commit 7 / manpower_app/utils.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>After XLS processing — why is 'add a job family' visible?</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Done (Target mode only)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Button now only appears when 'Input and Optimize a Target Manpower Plan' is selected, with a short hint explaining the flow. Hidden in Current mode — adding a family with no payroll rows has nothing to optimize.</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>commit 6 / MappingResolveWorkspace.tsx + App.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Make Outsourceable / Fully Inhouse / Partially Outsourceable dynamic</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Deferred (discussion)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Currently hardcoded in manpower_app/rules.py. Backend rework required: source (workbook column vs in-app editor), API contract, propagation through rules/costs/LP.</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>follow-up PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Saudis-cheaper-than-non-Saudis (auto-correct)</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Saudi cost premium floored at 1.0× in three places (defense in depth): desktop slider min, manpower_api Pydantic validator, and manpower_app.costs.calculate_inhouse_cost_split. Saudis can no longer be configured as cheaper than non-Saudis from any code path.</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>commit 4 / costs.py + ScenarioControls.tsx + app.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Hard inputs — edit ratio AND driver name (e.g., quarries labor vs skilled labor)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Deferred (discussion)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Driver mappings are hardcoded in manpower_app/ratios.py:calculate_driver_values. Same backend pattern as the dynamic-outsourceability item: new settings field, new API contract, propagation through the LP. Best done with the previous item.</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>follow-up PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Target plan — ask about drivers so ratios can be recalculated</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Deferred (discussion)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Depends on the editable-driver work above. Once a user can pin which profession is the ratio driver, the target plan UI needs an input for the driver headcount.</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>follow-up PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>Debugging</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Risk input slider — should reach zero</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Slider min lowered from 0.01 to 0 in UI and API. At R=0 the LP constraint degenerates cleanly to O+I ≥ M; the rearranged closed-form (T−M)/R is only consulted when R&gt;0. README updated.</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>commit 4 / ScenarioControls.tsx + app.py + README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Debugging</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>All tabs — '0' doesn't get deleted in number inputs</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Replaced controlled &lt;input type='number'&gt; with NumericTextInput (type='text' + inputMode='decimal') backed by an internal text buffer. On focus the value is selected; first keystroke replaces 0 cleanly across all browsers. Also accepts optional value/placeholder so the target-headcount field can show empty + a 'current headcount' placeholder.</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Replaced controlled &lt;input type='number'&gt; with NumericTextInput (type='text' + inputMode='decimal') backed by a text buffer. First keystroke replaces 0 cleanly. Supports optional value/placeholder for the target-headcount field.</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>commits 5 + 6 / ScenarioControls.tsx</t>
         </is>
@@ -1245,7 +1461,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1256,7 +1472,7 @@
       </c>
       <c r="B1" s="8" t="inlineStr">
         <is>
-          <t>150526_Manpower Optimization Tool Enhancements.xlsx</t>
+          <t>150526_Manpower Optimization Tool Enhancements (1).xlsx</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1519,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -1313,7 +1529,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
@@ -1404,14 +1620,14 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Net-new workflow stage. Spec hints 'after homepage, list of companies, click MGIC' but the same line flags the assumption risk: 'they will always run the app on one laptop'. Needs a design pass.</t>
+          <t>Net-new workflow stage. Spec hints 'after homepage, list of companies, click MGIC' but the same line flags the assumption risk: 'they will always run the app on one laptop'.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>1. Where does BU Selection sit in the workflow (before upload, after upload, side-panel)?
 2. Is the company list driven by data (a config workbook?) or hardcoded?
-3. Do we need per-BU data persistence (different workbooks loaded per BU)?
+3. Do we need per-BU data persistence?
 4. Multi-user / multi-machine collaboration implications.</t>
         </is>
       </c>
@@ -1441,14 +1657,14 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Currently OUTSOURCEABILITY_RULES is hardcoded across 40 job families in manpower_app/rules.py. Making this dynamic affects rules → costs → optimization constraints.</t>
+          <t>Currently OUTSOURCEABILITY_RULES is hardcoded across 40 job families in manpower_app/rules.py. Affects rules → costs → optimization constraints.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>1. Source: workbook column, in-app editor, or both?
 2. Per-BU overrides (ties into #4)?
-3. Validation: how to prevent inconsistent states (Fully Outsourceable + a non-zero ratio override)?</t>
+3. Validation: prevent inconsistent states (Fully Outsourceable + a non-zero ratio override).</t>
         </is>
       </c>
     </row>
@@ -1465,8 +1681,8 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>1. UI: free-text label vs structured (activity + profession) picker?
-2. Backend: new settings field driver_overrides — needs propagation through calculate_driver_values, the API, and the LP.
+          <t>1. UI: free-text label vs structured picker (activity + profession)?
+2. Backend: new settings field driver_overrides — needs propagation through calculate_driver_values, API, and LP.
 3. Should this share data with the partial-config 'driver-based' option in the custom-family wizard?</t>
         </is>
       </c>
@@ -1479,7 +1695,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Requires #22 first. Once driver is editable, the target plan needs an input field for the driver headcount so ratios can be recalculated from the user's target.</t>
+          <t>Requires editable drivers (#22) first. Then the target plan needs an input field for the driver headcount so ratios can be recalculated.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1496,13 +1712,13 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>All changes in this PR target the Desktop React UI. Streamlit (manpower_app/ui_streamlit.py) was deliberately left out of scope.</t>
+          <t>All changes in this PR target the Desktop React UI. Streamlit (manpower_app/ui_streamlit.py) is deliberately out of scope.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>1. Is Streamlit still a supported delivery surface, or is it being sunsetted in favor of the Tauri desktop / web container?
-2. If kept: do we mirror these UI changes (significant effort) or only the backend changes?</t>
+2. If kept: do we mirror these UI changes (significant effort) or only backend changes?</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1730,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Code currently lives at github.com/BahaaKaaki/manpower-optimization, public. README points to pwc-me-adv-strategyand/manpower-optimization as the canonical source. The Manpower.xlsx in the repo contains employee-level data.</t>
+          <t>Code currently lives at github.com/BahaaKaaki/manpower-optimization (public). README points to pwc-me-adv-strategyand/manpower-optimization as canonical source. Manpower.xlsx in the repo contains employee-level data.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1531,12 +1747,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The 94s → 19s win is from caching only. Remaining cost breakdown (cProfile): ~14s pandas .apply(axis=1) row iteration across 14 separate passes, ~6s openpyxl reading the .xlsx.</t>
+          <t>The 94s → 19s win is caching only. Remaining cost: ~14s pandas .apply(axis=1) row iteration across 14 separate passes, ~6s openpyxl XML parsing.</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Two follow-up options:
+          <t>Options:
 1. Vectorize the cost calculations (replace row-wise apply with column-wise pandas ops). Bigger refactor, ~5-10× more savings on the apply path.
 2. Switch the Excel reader engine to calamine (python-calamine). One-line change in pipeline.py, ~3-5× speedup on the read path, adds one dependency.</t>
         </is>

</xml_diff>